<commit_message>
Cibles modifiées PAB FDS SIC
</commit_message>
<xml_diff>
--- a/tests/Cibles.xlsx
+++ b/tests/Cibles.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mayt8801\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MAYT8801\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -1079,10 +1079,10 @@
         <v>10</v>
       </c>
       <c r="H21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J21">
         <v>0</v>

</xml_diff>